<commit_message>
update des profils ePrescription suite à analyse comparative (#134) 7cc169b0de4e2cd6947e52f66642ace7eb5256f0
</commit_message>
<xml_diff>
--- a/main/ig/StructureDefinition-fr-medication-document.xlsx
+++ b/main/ig/StructureDefinition-fr-medication-document.xlsx
@@ -10,13 +10,13 @@
     <sheet name="Elements" r:id="rId4" sheetId="2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">Elements!$A$1:$AN$58</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">Elements!$A$1:$AN$46</definedName>
   </definedNames>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2115" uniqueCount="336">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1685" uniqueCount="317">
   <si>
     <t>Property</t>
   </si>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-05-06T07:44:21+00:00</t>
+    <t>2026-05-13T14:53:03+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -481,7 +481,7 @@
 </t>
   </si>
   <si>
-    <t>Équivalent générique (Code de regroupement ATC) et le Conditionnement (Code du produit de santé conditionné (CIP)).</t>
+    <t>Classification ATC.</t>
   </si>
   <si>
     <t>Medication classification/category. Allows the product to be classified by various systems, e.g ATC, narcotic class, legal status of supply, etc..</t>
@@ -630,7 +630,7 @@
 </t>
   </si>
   <si>
-    <t>Autres codifications (CIP, UCD, ATC, MV)</t>
+    <t>Code defined by a terminology system</t>
   </si>
   <si>
     <t>A reference to a code defined by a terminology system.</t>
@@ -785,10 +785,6 @@
     <t>The ingredients need not be a complete list.  If an ingredient is not specified, this does not indicate whether an ingredient is present or absent.  If an ingredient is specified it does not mean that all ingredients are specified.  It is possible to specify both inactive and active ingredients.</t>
   </si>
   <si>
-    <t xml:space="preserve">value:$this}
-</t>
-  </si>
-  <si>
     <t>.scopesRole[typeCode=INGR]</t>
   </si>
   <si>
@@ -831,10 +827,66 @@
     <t>The ingredient may reference a substance (for example, amoxicillin) or another medication (for example in the case of a compounded product, Glaxal Base).</t>
   </si>
   <si>
+    <t xml:space="preserve">type:$this}
+</t>
+  </si>
+  <si>
+    <t>closed</t>
+  </si>
+  <si>
     <t>.player</t>
   </si>
   <si>
     <t>RXC-2-Component Code  if medication: RXO-1-Requested Give Code / RXE-2-Give Code / RXD-2-Dispense/Give Code / RXG-4-Give Code / RXA-5-Administered Code</t>
+  </si>
+  <si>
+    <t>Medication.ingredient.item[x]:itemCodeableConcept</t>
+  </si>
+  <si>
+    <t>itemCodeableConcept</t>
+  </si>
+  <si>
+    <t>Code SMS de la substance active</t>
+  </si>
+  <si>
+    <t>https://smt.esante.gouv.fr/terminologie-sms?vs</t>
+  </si>
+  <si>
+    <t>Medication.ingredient.item[x]:itemCodeableConcept.id</t>
+  </si>
+  <si>
+    <t>Medication.ingredient.item[x].id</t>
+  </si>
+  <si>
+    <t>Medication.ingredient.item[x]:itemCodeableConcept.extension</t>
+  </si>
+  <si>
+    <t>Medication.ingredient.item[x].extension</t>
+  </si>
+  <si>
+    <t>Medication.ingredient.item[x]:itemCodeableConcept.coding</t>
+  </si>
+  <si>
+    <t>Medication.ingredient.item[x].coding</t>
+  </si>
+  <si>
+    <t>Medication.ingredient.item[x]:itemCodeableConcept.text</t>
+  </si>
+  <si>
+    <t>Medication.ingredient.item[x].text</t>
+  </si>
+  <si>
+    <t>Nom de la substance</t>
+  </si>
+  <si>
+    <t>Medication.ingredient.item[x]:itemReference</t>
+  </si>
+  <si>
+    <t>itemReference</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reference(https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/fr-medication-document)
+</t>
   </si>
   <si>
     <t>Medication.ingredient.isActive</t>
@@ -860,7 +912,7 @@
     <t>Medication.ingredient.strength</t>
   </si>
   <si>
-    <t>Quantity of ingredient present</t>
+    <t>Quantité de substance présente dans le médicament</t>
   </si>
   <si>
     <t>Specifies how many (or how much) of the items there are in this Medication.  For example, 250 mg per tablet.  This is expressed as a ratio where the numerator is 250mg and the denominator is 1 tablet.</t>
@@ -872,115 +924,10 @@
     <t>RXC-3-Component Amount &amp; RXC-4-Component Units  if medication: RXO-2-Requested Give Amount - Minimum &amp; RXO-4-Requested Give Units / RXO-3-Requested Give Amount - Maximum &amp; RXO-4-Requested Give Units / RXO-11-Requested Dispense Amount &amp; RXO-12-Requested Dispense Units / RXE-3-Give Amount - Minimum &amp; RXE-5-Give Units / RXE-4-Give Amount - Maximum &amp; RXE-5-Give Units / RXE-10-Dispense Amount &amp; RXE-10-Dispense Units</t>
   </si>
   <si>
-    <t>Medication.ingredient:doseAntigene</t>
-  </si>
-  <si>
-    <t>doseAntigene</t>
-  </si>
-  <si>
-    <t>Dose antigène</t>
-  </si>
-  <si>
-    <t>Medication.ingredient:doseAntigene.id</t>
-  </si>
-  <si>
-    <t>Medication.ingredient:doseAntigene.extension</t>
-  </si>
-  <si>
-    <t>Medication.ingredient:doseAntigene.modifierExtension</t>
-  </si>
-  <si>
-    <t>Medication.ingredient:doseAntigene.item[x]</t>
-  </si>
-  <si>
-    <t>Medication.ingredient:doseAntigene.isActive</t>
-  </si>
-  <si>
-    <t>Medication.ingredient:doseAntigene.strength</t>
-  </si>
-  <si>
-    <t>Quantité de la dose antigène</t>
-  </si>
-  <si>
-    <t>Medication.ingredient:substanceActive</t>
-  </si>
-  <si>
-    <t>substanceActive</t>
-  </si>
-  <si>
-    <t>Substance active</t>
-  </si>
-  <si>
-    <t>Medication.ingredient:substanceActive.id</t>
-  </si>
-  <si>
-    <t>Medication.ingredient:substanceActive.extension</t>
-  </si>
-  <si>
-    <t>Medication.ingredient:substanceActive.modifierExtension</t>
-  </si>
-  <si>
-    <t>Medication.ingredient:substanceActive.item[x]</t>
-  </si>
-  <si>
-    <t>Code SMS de la substance active</t>
-  </si>
-  <si>
-    <t>https://smt.esante.gouv.fr/terminologie-sms?vs</t>
-  </si>
-  <si>
-    <t>Medication.ingredient:substanceActive.item[x].id</t>
-  </si>
-  <si>
-    <t>Medication.ingredient.item[x].id</t>
-  </si>
-  <si>
-    <t>Medication.ingredient:substanceActive.item[x].extension</t>
-  </si>
-  <si>
-    <t>Medication.ingredient.item[x].extension</t>
-  </si>
-  <si>
-    <t>Medication.ingredient:substanceActive.item[x].coding</t>
-  </si>
-  <si>
-    <t>Medication.ingredient.item[x].coding</t>
-  </si>
-  <si>
-    <t>Code defined by a terminology system</t>
-  </si>
-  <si>
-    <t>Medication.ingredient:substanceActive.item[x].text</t>
-  </si>
-  <si>
-    <t>Medication.ingredient.item[x].text</t>
-  </si>
-  <si>
-    <t>Nom de la substance</t>
-  </si>
-  <si>
-    <t>Medication.ingredient:substanceActive.isActive</t>
-  </si>
-  <si>
-    <t>Medication.ingredient:substanceActive.strength</t>
-  </si>
-  <si>
-    <t>Dosage</t>
-  </si>
-  <si>
-    <t>Medication.ingredient:substanceActive.strength.id</t>
-  </si>
-  <si>
     <t>Medication.ingredient.strength.id</t>
   </si>
   <si>
-    <t>Medication.ingredient:substanceActive.strength.extension</t>
-  </si>
-  <si>
     <t>Medication.ingredient.strength.extension</t>
-  </si>
-  <si>
-    <t>Medication.ingredient:substanceActive.strength.numerator</t>
   </si>
   <si>
     <t>Medication.ingredient.strength.numerator</t>
@@ -1000,9 +947,6 @@
   </si>
   <si>
     <t>.numerator</t>
-  </si>
-  <si>
-    <t>Medication.ingredient:substanceActive.strength.denominator</t>
   </si>
   <si>
     <t>Medication.ingredient.strength.denominator</t>
@@ -1386,12 +1330,12 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:AN58"/>
+  <dimension ref="A1:AN46"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" width="49.234375" customWidth="true" bestFit="true"/>
+    <col min="1" max="1" width="50.4140625" customWidth="true" bestFit="true"/>
     <col min="2" max="2" width="35.77734375" customWidth="true" bestFit="true"/>
-    <col min="3" max="3" width="14.234375" customWidth="true" bestFit="true" hidden="true"/>
+    <col min="3" max="3" width="18.3359375" customWidth="true" bestFit="true" hidden="true"/>
     <col min="4" max="4" width="34.21875" customWidth="true" bestFit="true" hidden="true"/>
     <col min="5" max="5" width="5.80859375" customWidth="true" bestFit="true"/>
     <col min="6" max="6" width="4.23828125" customWidth="true" bestFit="true"/>
@@ -1399,7 +1343,7 @@
     <col min="8" max="8" width="13.953125" customWidth="true" bestFit="true"/>
     <col min="9" max="9" width="11.3671875" customWidth="true" bestFit="true"/>
     <col min="10" max="10" width="20.703125" customWidth="true" bestFit="true"/>
-    <col min="11" max="11" width="80.8671875" customWidth="true" bestFit="true"/>
+    <col min="11" max="11" width="82.75390625" customWidth="true" bestFit="true"/>
     <col min="12" max="12" width="100.703125" customWidth="true" bestFit="true"/>
     <col min="13" max="13" width="100.703125" customWidth="true" bestFit="true"/>
     <col min="14" max="14" width="100.703125" customWidth="true" bestFit="true"/>
@@ -4061,7 +4005,7 @@
       </c>
       <c r="E24" s="2"/>
       <c r="F24" t="s" s="2">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="G24" t="s" s="2">
         <v>79</v>
@@ -4123,14 +4067,16 @@
         <v>77</v>
       </c>
       <c r="AB24" t="s" s="2">
-        <v>243</v>
-      </c>
-      <c r="AC24" s="2"/>
+        <v>77</v>
+      </c>
+      <c r="AC24" t="s" s="2">
+        <v>77</v>
+      </c>
       <c r="AD24" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AE24" t="s" s="2">
-        <v>136</v>
+        <v>77</v>
       </c>
       <c r="AF24" t="s" s="2">
         <v>238</v>
@@ -4151,7 +4097,7 @@
         <v>77</v>
       </c>
       <c r="AL24" t="s" s="2">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="AM24" t="s" s="2">
         <v>77</v>
@@ -4162,10 +4108,10 @@
     </row>
     <row r="25" hidden="true">
       <c r="A25" t="s" s="2">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="B25" t="s" s="2">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="C25" s="2"/>
       <c r="D25" t="s" s="2">
@@ -4274,10 +4220,10 @@
     </row>
     <row r="26" hidden="true">
       <c r="A26" t="s" s="2">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B26" t="s" s="2">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="C26" s="2"/>
       <c r="D26" t="s" s="2">
@@ -4388,14 +4334,14 @@
     </row>
     <row r="27" hidden="true">
       <c r="A27" t="s" s="2">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="B27" t="s" s="2">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="C27" s="2"/>
       <c r="D27" t="s" s="2">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="E27" s="2"/>
       <c r="F27" t="s" s="2">
@@ -4417,10 +4363,10 @@
         <v>132</v>
       </c>
       <c r="L27" t="s" s="2">
+        <v>248</v>
+      </c>
+      <c r="M27" t="s" s="2">
         <v>249</v>
-      </c>
-      <c r="M27" t="s" s="2">
-        <v>250</v>
       </c>
       <c r="N27" t="s" s="2">
         <v>158</v>
@@ -4475,7 +4421,7 @@
         <v>77</v>
       </c>
       <c r="AF27" t="s" s="2">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="AG27" t="s" s="2">
         <v>78</v>
@@ -4504,10 +4450,10 @@
     </row>
     <row r="28" hidden="true">
       <c r="A28" t="s" s="2">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="B28" t="s" s="2">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="C28" s="2"/>
       <c r="D28" t="s" s="2">
@@ -4530,17 +4476,17 @@
         <v>77</v>
       </c>
       <c r="K28" t="s" s="2">
+        <v>252</v>
+      </c>
+      <c r="L28" t="s" s="2">
         <v>253</v>
       </c>
-      <c r="L28" t="s" s="2">
+      <c r="M28" t="s" s="2">
         <v>254</v>
-      </c>
-      <c r="M28" t="s" s="2">
-        <v>255</v>
       </c>
       <c r="N28" s="2"/>
       <c r="O28" t="s" s="2">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="P28" t="s" s="2">
         <v>77</v>
@@ -4577,19 +4523,17 @@
         <v>77</v>
       </c>
       <c r="AB28" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AC28" t="s" s="2">
-        <v>77</v>
-      </c>
+        <v>256</v>
+      </c>
+      <c r="AC28" s="2"/>
       <c r="AD28" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AE28" t="s" s="2">
-        <v>77</v>
+        <v>257</v>
       </c>
       <c r="AF28" t="s" s="2">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="AG28" t="s" s="2">
         <v>87</v>
@@ -4607,23 +4551,25 @@
         <v>176</v>
       </c>
       <c r="AL28" t="s" s="2">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="AM28" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AN28" t="s" s="2">
-        <v>258</v>
+        <v>259</v>
       </c>
     </row>
-    <row r="29" hidden="true">
+    <row r="29">
       <c r="A29" t="s" s="2">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="B29" t="s" s="2">
-        <v>259</v>
-      </c>
-      <c r="C29" s="2"/>
+        <v>251</v>
+      </c>
+      <c r="C29" t="s" s="2">
+        <v>261</v>
+      </c>
       <c r="D29" t="s" s="2">
         <v>77</v>
       </c>
@@ -4635,7 +4581,7 @@
         <v>87</v>
       </c>
       <c r="H29" t="s" s="2">
-        <v>77</v>
+        <v>88</v>
       </c>
       <c r="I29" t="s" s="2">
         <v>77</v>
@@ -4644,17 +4590,17 @@
         <v>77</v>
       </c>
       <c r="K29" t="s" s="2">
-        <v>260</v>
+        <v>169</v>
       </c>
       <c r="L29" t="s" s="2">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="M29" t="s" s="2">
-        <v>262</v>
+        <v>254</v>
       </c>
       <c r="N29" s="2"/>
       <c r="O29" t="s" s="2">
-        <v>263</v>
+        <v>255</v>
       </c>
       <c r="P29" t="s" s="2">
         <v>77</v>
@@ -4679,13 +4625,11 @@
         <v>77</v>
       </c>
       <c r="X29" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="Y29" t="s" s="2">
-        <v>77</v>
-      </c>
+        <v>197</v>
+      </c>
+      <c r="Y29" s="2"/>
       <c r="Z29" t="s" s="2">
-        <v>77</v>
+        <v>263</v>
       </c>
       <c r="AA29" t="s" s="2">
         <v>77</v>
@@ -4703,10 +4647,10 @@
         <v>77</v>
       </c>
       <c r="AF29" t="s" s="2">
-        <v>259</v>
+        <v>251</v>
       </c>
       <c r="AG29" t="s" s="2">
-        <v>78</v>
+        <v>87</v>
       </c>
       <c r="AH29" t="s" s="2">
         <v>87</v>
@@ -4718,21 +4662,21 @@
         <v>99</v>
       </c>
       <c r="AK29" t="s" s="2">
-        <v>77</v>
+        <v>176</v>
       </c>
       <c r="AL29" t="s" s="2">
-        <v>264</v>
+        <v>258</v>
       </c>
       <c r="AM29" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AN29" t="s" s="2">
-        <v>77</v>
+        <v>259</v>
       </c>
     </row>
     <row r="30" hidden="true">
       <c r="A30" t="s" s="2">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="B30" t="s" s="2">
         <v>265</v>
@@ -4758,13 +4702,13 @@
         <v>77</v>
       </c>
       <c r="K30" t="s" s="2">
-        <v>234</v>
+        <v>181</v>
       </c>
       <c r="L30" t="s" s="2">
-        <v>266</v>
+        <v>182</v>
       </c>
       <c r="M30" t="s" s="2">
-        <v>267</v>
+        <v>183</v>
       </c>
       <c r="N30" s="2"/>
       <c r="O30" s="2"/>
@@ -4815,7 +4759,7 @@
         <v>77</v>
       </c>
       <c r="AF30" t="s" s="2">
-        <v>265</v>
+        <v>184</v>
       </c>
       <c r="AG30" t="s" s="2">
         <v>78</v>
@@ -4827,33 +4771,31 @@
         <v>77</v>
       </c>
       <c r="AJ30" t="s" s="2">
-        <v>99</v>
+        <v>77</v>
       </c>
       <c r="AK30" t="s" s="2">
-        <v>268</v>
+        <v>77</v>
       </c>
       <c r="AL30" t="s" s="2">
-        <v>237</v>
+        <v>185</v>
       </c>
       <c r="AM30" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AN30" t="s" s="2">
-        <v>269</v>
+        <v>77</v>
       </c>
     </row>
-    <row r="31">
+    <row r="31" hidden="true">
       <c r="A31" t="s" s="2">
-        <v>270</v>
+        <v>266</v>
       </c>
       <c r="B31" t="s" s="2">
-        <v>238</v>
-      </c>
-      <c r="C31" t="s" s="2">
-        <v>271</v>
-      </c>
+        <v>267</v>
+      </c>
+      <c r="C31" s="2"/>
       <c r="D31" t="s" s="2">
-        <v>77</v>
+        <v>155</v>
       </c>
       <c r="E31" s="2"/>
       <c r="F31" t="s" s="2">
@@ -4863,7 +4805,7 @@
         <v>79</v>
       </c>
       <c r="H31" t="s" s="2">
-        <v>88</v>
+        <v>77</v>
       </c>
       <c r="I31" t="s" s="2">
         <v>77</v>
@@ -4872,16 +4814,16 @@
         <v>77</v>
       </c>
       <c r="K31" t="s" s="2">
-        <v>239</v>
+        <v>132</v>
       </c>
       <c r="L31" t="s" s="2">
-        <v>272</v>
+        <v>187</v>
       </c>
       <c r="M31" t="s" s="2">
-        <v>241</v>
+        <v>188</v>
       </c>
       <c r="N31" t="s" s="2">
-        <v>242</v>
+        <v>158</v>
       </c>
       <c r="O31" s="2"/>
       <c r="P31" t="s" s="2">
@@ -4919,19 +4861,19 @@
         <v>77</v>
       </c>
       <c r="AB31" t="s" s="2">
-        <v>77</v>
+        <v>135</v>
       </c>
       <c r="AC31" t="s" s="2">
-        <v>77</v>
+        <v>189</v>
       </c>
       <c r="AD31" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AE31" t="s" s="2">
-        <v>77</v>
+        <v>136</v>
       </c>
       <c r="AF31" t="s" s="2">
-        <v>238</v>
+        <v>190</v>
       </c>
       <c r="AG31" t="s" s="2">
         <v>78</v>
@@ -4943,13 +4885,13 @@
         <v>77</v>
       </c>
       <c r="AJ31" t="s" s="2">
-        <v>99</v>
+        <v>138</v>
       </c>
       <c r="AK31" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AL31" t="s" s="2">
-        <v>244</v>
+        <v>185</v>
       </c>
       <c r="AM31" t="s" s="2">
         <v>77</v>
@@ -4960,10 +4902,10 @@
     </row>
     <row r="32" hidden="true">
       <c r="A32" t="s" s="2">
-        <v>273</v>
+        <v>268</v>
       </c>
       <c r="B32" t="s" s="2">
-        <v>245</v>
+        <v>269</v>
       </c>
       <c r="C32" s="2"/>
       <c r="D32" t="s" s="2">
@@ -4974,7 +4916,7 @@
         <v>78</v>
       </c>
       <c r="G32" t="s" s="2">
-        <v>87</v>
+        <v>79</v>
       </c>
       <c r="H32" t="s" s="2">
         <v>77</v>
@@ -4983,19 +4925,23 @@
         <v>77</v>
       </c>
       <c r="J32" t="s" s="2">
-        <v>77</v>
+        <v>88</v>
       </c>
       <c r="K32" t="s" s="2">
-        <v>181</v>
+        <v>192</v>
       </c>
       <c r="L32" t="s" s="2">
-        <v>182</v>
+        <v>193</v>
       </c>
       <c r="M32" t="s" s="2">
-        <v>183</v>
-      </c>
-      <c r="N32" s="2"/>
-      <c r="O32" s="2"/>
+        <v>194</v>
+      </c>
+      <c r="N32" t="s" s="2">
+        <v>195</v>
+      </c>
+      <c r="O32" t="s" s="2">
+        <v>196</v>
+      </c>
       <c r="P32" t="s" s="2">
         <v>77</v>
       </c>
@@ -5043,73 +4989,75 @@
         <v>77</v>
       </c>
       <c r="AF32" t="s" s="2">
-        <v>184</v>
+        <v>199</v>
       </c>
       <c r="AG32" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH32" t="s" s="2">
-        <v>87</v>
+        <v>79</v>
       </c>
       <c r="AI32" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AJ32" t="s" s="2">
-        <v>77</v>
+        <v>99</v>
       </c>
       <c r="AK32" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AL32" t="s" s="2">
-        <v>185</v>
+        <v>200</v>
       </c>
       <c r="AM32" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AN32" t="s" s="2">
-        <v>77</v>
+        <v>201</v>
       </c>
     </row>
-    <row r="33" hidden="true">
+    <row r="33">
       <c r="A33" t="s" s="2">
-        <v>274</v>
+        <v>270</v>
       </c>
       <c r="B33" t="s" s="2">
-        <v>246</v>
+        <v>271</v>
       </c>
       <c r="C33" s="2"/>
       <c r="D33" t="s" s="2">
-        <v>155</v>
+        <v>77</v>
       </c>
       <c r="E33" s="2"/>
       <c r="F33" t="s" s="2">
         <v>78</v>
       </c>
       <c r="G33" t="s" s="2">
-        <v>79</v>
+        <v>87</v>
       </c>
       <c r="H33" t="s" s="2">
-        <v>77</v>
+        <v>88</v>
       </c>
       <c r="I33" t="s" s="2">
         <v>77</v>
       </c>
       <c r="J33" t="s" s="2">
-        <v>77</v>
+        <v>88</v>
       </c>
       <c r="K33" t="s" s="2">
-        <v>132</v>
+        <v>181</v>
       </c>
       <c r="L33" t="s" s="2">
-        <v>187</v>
+        <v>272</v>
       </c>
       <c r="M33" t="s" s="2">
-        <v>188</v>
+        <v>204</v>
       </c>
       <c r="N33" t="s" s="2">
-        <v>158</v>
-      </c>
-      <c r="O33" s="2"/>
+        <v>205</v>
+      </c>
+      <c r="O33" t="s" s="2">
+        <v>206</v>
+      </c>
       <c r="P33" t="s" s="2">
         <v>77</v>
       </c>
@@ -5157,74 +5105,74 @@
         <v>77</v>
       </c>
       <c r="AF33" t="s" s="2">
-        <v>190</v>
+        <v>207</v>
       </c>
       <c r="AG33" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH33" t="s" s="2">
-        <v>79</v>
+        <v>87</v>
       </c>
       <c r="AI33" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AJ33" t="s" s="2">
-        <v>138</v>
+        <v>99</v>
       </c>
       <c r="AK33" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AL33" t="s" s="2">
-        <v>185</v>
+        <v>208</v>
       </c>
       <c r="AM33" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AN33" t="s" s="2">
-        <v>77</v>
+        <v>209</v>
       </c>
     </row>
-    <row r="34" hidden="true">
+    <row r="34">
       <c r="A34" t="s" s="2">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="B34" t="s" s="2">
-        <v>247</v>
-      </c>
-      <c r="C34" s="2"/>
+        <v>251</v>
+      </c>
+      <c r="C34" t="s" s="2">
+        <v>274</v>
+      </c>
       <c r="D34" t="s" s="2">
-        <v>248</v>
+        <v>77</v>
       </c>
       <c r="E34" s="2"/>
       <c r="F34" t="s" s="2">
         <v>78</v>
       </c>
       <c r="G34" t="s" s="2">
-        <v>79</v>
+        <v>87</v>
       </c>
       <c r="H34" t="s" s="2">
-        <v>77</v>
+        <v>88</v>
       </c>
       <c r="I34" t="s" s="2">
-        <v>88</v>
+        <v>77</v>
       </c>
       <c r="J34" t="s" s="2">
-        <v>88</v>
+        <v>77</v>
       </c>
       <c r="K34" t="s" s="2">
-        <v>132</v>
+        <v>275</v>
       </c>
       <c r="L34" t="s" s="2">
-        <v>249</v>
+        <v>253</v>
       </c>
       <c r="M34" t="s" s="2">
-        <v>250</v>
-      </c>
-      <c r="N34" t="s" s="2">
-        <v>158</v>
-      </c>
+        <v>254</v>
+      </c>
+      <c r="N34" s="2"/>
       <c r="O34" t="s" s="2">
-        <v>159</v>
+        <v>255</v>
       </c>
       <c r="P34" t="s" s="2">
         <v>77</v>
@@ -5276,28 +5224,28 @@
         <v>251</v>
       </c>
       <c r="AG34" t="s" s="2">
-        <v>78</v>
+        <v>87</v>
       </c>
       <c r="AH34" t="s" s="2">
-        <v>79</v>
+        <v>87</v>
       </c>
       <c r="AI34" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AJ34" t="s" s="2">
-        <v>138</v>
+        <v>99</v>
       </c>
       <c r="AK34" t="s" s="2">
-        <v>77</v>
+        <v>176</v>
       </c>
       <c r="AL34" t="s" s="2">
-        <v>130</v>
+        <v>258</v>
       </c>
       <c r="AM34" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AN34" t="s" s="2">
-        <v>77</v>
+        <v>259</v>
       </c>
     </row>
     <row r="35" hidden="true">
@@ -5305,7 +5253,7 @@
         <v>276</v>
       </c>
       <c r="B35" t="s" s="2">
-        <v>252</v>
+        <v>276</v>
       </c>
       <c r="C35" s="2"/>
       <c r="D35" t="s" s="2">
@@ -5313,7 +5261,7 @@
       </c>
       <c r="E35" s="2"/>
       <c r="F35" t="s" s="2">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="G35" t="s" s="2">
         <v>87</v>
@@ -5328,17 +5276,17 @@
         <v>77</v>
       </c>
       <c r="K35" t="s" s="2">
-        <v>253</v>
+        <v>277</v>
       </c>
       <c r="L35" t="s" s="2">
-        <v>254</v>
+        <v>278</v>
       </c>
       <c r="M35" t="s" s="2">
-        <v>255</v>
+        <v>279</v>
       </c>
       <c r="N35" s="2"/>
       <c r="O35" t="s" s="2">
-        <v>256</v>
+        <v>280</v>
       </c>
       <c r="P35" t="s" s="2">
         <v>77</v>
@@ -5387,10 +5335,10 @@
         <v>77</v>
       </c>
       <c r="AF35" t="s" s="2">
-        <v>252</v>
+        <v>276</v>
       </c>
       <c r="AG35" t="s" s="2">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="AH35" t="s" s="2">
         <v>87</v>
@@ -5402,24 +5350,24 @@
         <v>99</v>
       </c>
       <c r="AK35" t="s" s="2">
-        <v>176</v>
+        <v>77</v>
       </c>
       <c r="AL35" t="s" s="2">
-        <v>257</v>
+        <v>281</v>
       </c>
       <c r="AM35" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AN35" t="s" s="2">
-        <v>258</v>
+        <v>77</v>
       </c>
     </row>
-    <row r="36" hidden="true">
+    <row r="36">
       <c r="A36" t="s" s="2">
-        <v>277</v>
+        <v>282</v>
       </c>
       <c r="B36" t="s" s="2">
-        <v>259</v>
+        <v>282</v>
       </c>
       <c r="C36" s="2"/>
       <c r="D36" t="s" s="2">
@@ -5433,7 +5381,7 @@
         <v>87</v>
       </c>
       <c r="H36" t="s" s="2">
-        <v>77</v>
+        <v>88</v>
       </c>
       <c r="I36" t="s" s="2">
         <v>77</v>
@@ -5442,18 +5390,16 @@
         <v>77</v>
       </c>
       <c r="K36" t="s" s="2">
-        <v>260</v>
+        <v>234</v>
       </c>
       <c r="L36" t="s" s="2">
-        <v>261</v>
+        <v>283</v>
       </c>
       <c r="M36" t="s" s="2">
-        <v>262</v>
+        <v>284</v>
       </c>
       <c r="N36" s="2"/>
-      <c r="O36" t="s" s="2">
-        <v>263</v>
-      </c>
+      <c r="O36" s="2"/>
       <c r="P36" t="s" s="2">
         <v>77</v>
       </c>
@@ -5501,7 +5447,7 @@
         <v>77</v>
       </c>
       <c r="AF36" t="s" s="2">
-        <v>259</v>
+        <v>282</v>
       </c>
       <c r="AG36" t="s" s="2">
         <v>78</v>
@@ -5516,24 +5462,24 @@
         <v>99</v>
       </c>
       <c r="AK36" t="s" s="2">
-        <v>77</v>
+        <v>285</v>
       </c>
       <c r="AL36" t="s" s="2">
-        <v>264</v>
+        <v>237</v>
       </c>
       <c r="AM36" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AN36" t="s" s="2">
-        <v>77</v>
+        <v>286</v>
       </c>
     </row>
-    <row r="37">
+    <row r="37" hidden="true">
       <c r="A37" t="s" s="2">
-        <v>278</v>
+        <v>287</v>
       </c>
       <c r="B37" t="s" s="2">
-        <v>265</v>
+        <v>287</v>
       </c>
       <c r="C37" s="2"/>
       <c r="D37" t="s" s="2">
@@ -5547,7 +5493,7 @@
         <v>87</v>
       </c>
       <c r="H37" t="s" s="2">
-        <v>88</v>
+        <v>77</v>
       </c>
       <c r="I37" t="s" s="2">
         <v>77</v>
@@ -5556,13 +5502,13 @@
         <v>77</v>
       </c>
       <c r="K37" t="s" s="2">
-        <v>234</v>
+        <v>181</v>
       </c>
       <c r="L37" t="s" s="2">
-        <v>279</v>
+        <v>182</v>
       </c>
       <c r="M37" t="s" s="2">
-        <v>267</v>
+        <v>183</v>
       </c>
       <c r="N37" s="2"/>
       <c r="O37" s="2"/>
@@ -5613,7 +5559,7 @@
         <v>77</v>
       </c>
       <c r="AF37" t="s" s="2">
-        <v>265</v>
+        <v>184</v>
       </c>
       <c r="AG37" t="s" s="2">
         <v>78</v>
@@ -5625,43 +5571,41 @@
         <v>77</v>
       </c>
       <c r="AJ37" t="s" s="2">
-        <v>99</v>
+        <v>77</v>
       </c>
       <c r="AK37" t="s" s="2">
-        <v>268</v>
+        <v>77</v>
       </c>
       <c r="AL37" t="s" s="2">
-        <v>237</v>
+        <v>185</v>
       </c>
       <c r="AM37" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AN37" t="s" s="2">
-        <v>269</v>
+        <v>77</v>
       </c>
     </row>
-    <row r="38">
+    <row r="38" hidden="true">
       <c r="A38" t="s" s="2">
-        <v>280</v>
+        <v>288</v>
       </c>
       <c r="B38" t="s" s="2">
-        <v>238</v>
-      </c>
-      <c r="C38" t="s" s="2">
-        <v>281</v>
-      </c>
+        <v>288</v>
+      </c>
+      <c r="C38" s="2"/>
       <c r="D38" t="s" s="2">
-        <v>77</v>
+        <v>155</v>
       </c>
       <c r="E38" s="2"/>
       <c r="F38" t="s" s="2">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="G38" t="s" s="2">
-        <v>87</v>
+        <v>79</v>
       </c>
       <c r="H38" t="s" s="2">
-        <v>88</v>
+        <v>77</v>
       </c>
       <c r="I38" t="s" s="2">
         <v>77</v>
@@ -5670,16 +5614,16 @@
         <v>77</v>
       </c>
       <c r="K38" t="s" s="2">
-        <v>239</v>
+        <v>132</v>
       </c>
       <c r="L38" t="s" s="2">
-        <v>282</v>
+        <v>187</v>
       </c>
       <c r="M38" t="s" s="2">
-        <v>241</v>
+        <v>188</v>
       </c>
       <c r="N38" t="s" s="2">
-        <v>242</v>
+        <v>158</v>
       </c>
       <c r="O38" s="2"/>
       <c r="P38" t="s" s="2">
@@ -5717,19 +5661,19 @@
         <v>77</v>
       </c>
       <c r="AB38" t="s" s="2">
-        <v>77</v>
+        <v>135</v>
       </c>
       <c r="AC38" t="s" s="2">
-        <v>77</v>
+        <v>189</v>
       </c>
       <c r="AD38" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AE38" t="s" s="2">
-        <v>77</v>
+        <v>136</v>
       </c>
       <c r="AF38" t="s" s="2">
-        <v>238</v>
+        <v>190</v>
       </c>
       <c r="AG38" t="s" s="2">
         <v>78</v>
@@ -5741,13 +5685,13 @@
         <v>77</v>
       </c>
       <c r="AJ38" t="s" s="2">
-        <v>99</v>
+        <v>138</v>
       </c>
       <c r="AK38" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AL38" t="s" s="2">
-        <v>244</v>
+        <v>185</v>
       </c>
       <c r="AM38" t="s" s="2">
         <v>77</v>
@@ -5756,12 +5700,12 @@
         <v>77</v>
       </c>
     </row>
-    <row r="39" hidden="true">
+    <row r="39">
       <c r="A39" t="s" s="2">
-        <v>283</v>
+        <v>289</v>
       </c>
       <c r="B39" t="s" s="2">
-        <v>245</v>
+        <v>289</v>
       </c>
       <c r="C39" s="2"/>
       <c r="D39" t="s" s="2">
@@ -5769,28 +5713,28 @@
       </c>
       <c r="E39" s="2"/>
       <c r="F39" t="s" s="2">
-        <v>78</v>
+        <v>87</v>
       </c>
       <c r="G39" t="s" s="2">
         <v>87</v>
       </c>
       <c r="H39" t="s" s="2">
-        <v>77</v>
+        <v>88</v>
       </c>
       <c r="I39" t="s" s="2">
         <v>77</v>
       </c>
       <c r="J39" t="s" s="2">
-        <v>77</v>
+        <v>88</v>
       </c>
       <c r="K39" t="s" s="2">
-        <v>181</v>
+        <v>290</v>
       </c>
       <c r="L39" t="s" s="2">
-        <v>182</v>
+        <v>291</v>
       </c>
       <c r="M39" t="s" s="2">
-        <v>183</v>
+        <v>292</v>
       </c>
       <c r="N39" s="2"/>
       <c r="O39" s="2"/>
@@ -5841,7 +5785,7 @@
         <v>77</v>
       </c>
       <c r="AF39" t="s" s="2">
-        <v>184</v>
+        <v>293</v>
       </c>
       <c r="AG39" t="s" s="2">
         <v>78</v>
@@ -5853,13 +5797,13 @@
         <v>77</v>
       </c>
       <c r="AJ39" t="s" s="2">
-        <v>77</v>
+        <v>99</v>
       </c>
       <c r="AK39" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AL39" t="s" s="2">
-        <v>185</v>
+        <v>294</v>
       </c>
       <c r="AM39" t="s" s="2">
         <v>77</v>
@@ -5868,45 +5812,43 @@
         <v>77</v>
       </c>
     </row>
-    <row r="40" hidden="true">
+    <row r="40">
       <c r="A40" t="s" s="2">
-        <v>284</v>
+        <v>295</v>
       </c>
       <c r="B40" t="s" s="2">
-        <v>246</v>
+        <v>295</v>
       </c>
       <c r="C40" s="2"/>
       <c r="D40" t="s" s="2">
-        <v>155</v>
+        <v>77</v>
       </c>
       <c r="E40" s="2"/>
       <c r="F40" t="s" s="2">
-        <v>78</v>
+        <v>87</v>
       </c>
       <c r="G40" t="s" s="2">
-        <v>79</v>
+        <v>87</v>
       </c>
       <c r="H40" t="s" s="2">
-        <v>77</v>
+        <v>88</v>
       </c>
       <c r="I40" t="s" s="2">
         <v>77</v>
       </c>
       <c r="J40" t="s" s="2">
-        <v>77</v>
+        <v>88</v>
       </c>
       <c r="K40" t="s" s="2">
-        <v>132</v>
+        <v>290</v>
       </c>
       <c r="L40" t="s" s="2">
-        <v>187</v>
+        <v>296</v>
       </c>
       <c r="M40" t="s" s="2">
-        <v>188</v>
-      </c>
-      <c r="N40" t="s" s="2">
-        <v>158</v>
-      </c>
+        <v>297</v>
+      </c>
+      <c r="N40" s="2"/>
       <c r="O40" s="2"/>
       <c r="P40" t="s" s="2">
         <v>77</v>
@@ -5955,25 +5897,25 @@
         <v>77</v>
       </c>
       <c r="AF40" t="s" s="2">
-        <v>190</v>
+        <v>298</v>
       </c>
       <c r="AG40" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH40" t="s" s="2">
-        <v>79</v>
+        <v>87</v>
       </c>
       <c r="AI40" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AJ40" t="s" s="2">
-        <v>138</v>
+        <v>99</v>
       </c>
       <c r="AK40" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AL40" t="s" s="2">
-        <v>185</v>
+        <v>299</v>
       </c>
       <c r="AM40" t="s" s="2">
         <v>77</v>
@@ -5984,46 +5926,42 @@
     </row>
     <row r="41" hidden="true">
       <c r="A41" t="s" s="2">
-        <v>285</v>
+        <v>300</v>
       </c>
       <c r="B41" t="s" s="2">
-        <v>247</v>
+        <v>300</v>
       </c>
       <c r="C41" s="2"/>
       <c r="D41" t="s" s="2">
-        <v>248</v>
+        <v>77</v>
       </c>
       <c r="E41" s="2"/>
       <c r="F41" t="s" s="2">
         <v>78</v>
       </c>
       <c r="G41" t="s" s="2">
-        <v>79</v>
+        <v>87</v>
       </c>
       <c r="H41" t="s" s="2">
         <v>77</v>
       </c>
       <c r="I41" t="s" s="2">
-        <v>88</v>
+        <v>77</v>
       </c>
       <c r="J41" t="s" s="2">
-        <v>88</v>
+        <v>77</v>
       </c>
       <c r="K41" t="s" s="2">
-        <v>132</v>
+        <v>239</v>
       </c>
       <c r="L41" t="s" s="2">
-        <v>249</v>
+        <v>301</v>
       </c>
       <c r="M41" t="s" s="2">
-        <v>250</v>
-      </c>
-      <c r="N41" t="s" s="2">
-        <v>158</v>
-      </c>
-      <c r="O41" t="s" s="2">
-        <v>159</v>
-      </c>
+        <v>302</v>
+      </c>
+      <c r="N41" s="2"/>
+      <c r="O41" s="2"/>
       <c r="P41" t="s" s="2">
         <v>77</v>
       </c>
@@ -6071,25 +6009,25 @@
         <v>77</v>
       </c>
       <c r="AF41" t="s" s="2">
-        <v>251</v>
+        <v>300</v>
       </c>
       <c r="AG41" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH41" t="s" s="2">
-        <v>79</v>
+        <v>87</v>
       </c>
       <c r="AI41" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AJ41" t="s" s="2">
-        <v>138</v>
+        <v>99</v>
       </c>
       <c r="AK41" t="s" s="2">
-        <v>77</v>
+        <v>221</v>
       </c>
       <c r="AL41" t="s" s="2">
-        <v>130</v>
+        <v>303</v>
       </c>
       <c r="AM41" t="s" s="2">
         <v>77</v>
@@ -6098,12 +6036,12 @@
         <v>77</v>
       </c>
     </row>
-    <row r="42">
+    <row r="42" hidden="true">
       <c r="A42" t="s" s="2">
-        <v>286</v>
+        <v>304</v>
       </c>
       <c r="B42" t="s" s="2">
-        <v>252</v>
+        <v>304</v>
       </c>
       <c r="C42" s="2"/>
       <c r="D42" t="s" s="2">
@@ -6111,13 +6049,13 @@
       </c>
       <c r="E42" s="2"/>
       <c r="F42" t="s" s="2">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="G42" t="s" s="2">
         <v>87</v>
       </c>
       <c r="H42" t="s" s="2">
-        <v>88</v>
+        <v>77</v>
       </c>
       <c r="I42" t="s" s="2">
         <v>77</v>
@@ -6126,18 +6064,16 @@
         <v>77</v>
       </c>
       <c r="K42" t="s" s="2">
-        <v>169</v>
+        <v>181</v>
       </c>
       <c r="L42" t="s" s="2">
-        <v>287</v>
+        <v>182</v>
       </c>
       <c r="M42" t="s" s="2">
-        <v>255</v>
+        <v>183</v>
       </c>
       <c r="N42" s="2"/>
-      <c r="O42" t="s" s="2">
-        <v>256</v>
-      </c>
+      <c r="O42" s="2"/>
       <c r="P42" t="s" s="2">
         <v>77</v>
       </c>
@@ -6161,11 +6097,13 @@
         <v>77</v>
       </c>
       <c r="X42" t="s" s="2">
-        <v>197</v>
-      </c>
-      <c r="Y42" s="2"/>
+        <v>77</v>
+      </c>
+      <c r="Y42" t="s" s="2">
+        <v>77</v>
+      </c>
       <c r="Z42" t="s" s="2">
-        <v>288</v>
+        <v>77</v>
       </c>
       <c r="AA42" t="s" s="2">
         <v>77</v>
@@ -6183,10 +6121,10 @@
         <v>77</v>
       </c>
       <c r="AF42" t="s" s="2">
-        <v>252</v>
+        <v>184</v>
       </c>
       <c r="AG42" t="s" s="2">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="AH42" t="s" s="2">
         <v>87</v>
@@ -6195,38 +6133,38 @@
         <v>77</v>
       </c>
       <c r="AJ42" t="s" s="2">
-        <v>99</v>
+        <v>77</v>
       </c>
       <c r="AK42" t="s" s="2">
-        <v>176</v>
+        <v>77</v>
       </c>
       <c r="AL42" t="s" s="2">
-        <v>257</v>
+        <v>185</v>
       </c>
       <c r="AM42" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AN42" t="s" s="2">
-        <v>258</v>
+        <v>77</v>
       </c>
     </row>
     <row r="43" hidden="true">
       <c r="A43" t="s" s="2">
-        <v>289</v>
+        <v>305</v>
       </c>
       <c r="B43" t="s" s="2">
-        <v>290</v>
+        <v>305</v>
       </c>
       <c r="C43" s="2"/>
       <c r="D43" t="s" s="2">
-        <v>77</v>
+        <v>155</v>
       </c>
       <c r="E43" s="2"/>
       <c r="F43" t="s" s="2">
         <v>78</v>
       </c>
       <c r="G43" t="s" s="2">
-        <v>87</v>
+        <v>79</v>
       </c>
       <c r="H43" t="s" s="2">
         <v>77</v>
@@ -6238,15 +6176,17 @@
         <v>77</v>
       </c>
       <c r="K43" t="s" s="2">
-        <v>181</v>
+        <v>132</v>
       </c>
       <c r="L43" t="s" s="2">
-        <v>182</v>
+        <v>187</v>
       </c>
       <c r="M43" t="s" s="2">
-        <v>183</v>
-      </c>
-      <c r="N43" s="2"/>
+        <v>188</v>
+      </c>
+      <c r="N43" t="s" s="2">
+        <v>158</v>
+      </c>
       <c r="O43" s="2"/>
       <c r="P43" t="s" s="2">
         <v>77</v>
@@ -6295,19 +6235,19 @@
         <v>77</v>
       </c>
       <c r="AF43" t="s" s="2">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="AG43" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH43" t="s" s="2">
-        <v>87</v>
+        <v>79</v>
       </c>
       <c r="AI43" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AJ43" t="s" s="2">
-        <v>77</v>
+        <v>138</v>
       </c>
       <c r="AK43" t="s" s="2">
         <v>77</v>
@@ -6324,14 +6264,14 @@
     </row>
     <row r="44" hidden="true">
       <c r="A44" t="s" s="2">
-        <v>291</v>
+        <v>306</v>
       </c>
       <c r="B44" t="s" s="2">
-        <v>292</v>
+        <v>306</v>
       </c>
       <c r="C44" s="2"/>
       <c r="D44" t="s" s="2">
-        <v>155</v>
+        <v>247</v>
       </c>
       <c r="E44" s="2"/>
       <c r="F44" t="s" s="2">
@@ -6344,24 +6284,26 @@
         <v>77</v>
       </c>
       <c r="I44" t="s" s="2">
-        <v>77</v>
+        <v>88</v>
       </c>
       <c r="J44" t="s" s="2">
-        <v>77</v>
+        <v>88</v>
       </c>
       <c r="K44" t="s" s="2">
         <v>132</v>
       </c>
       <c r="L44" t="s" s="2">
-        <v>187</v>
+        <v>248</v>
       </c>
       <c r="M44" t="s" s="2">
-        <v>188</v>
+        <v>249</v>
       </c>
       <c r="N44" t="s" s="2">
         <v>158</v>
       </c>
-      <c r="O44" s="2"/>
+      <c r="O44" t="s" s="2">
+        <v>159</v>
+      </c>
       <c r="P44" t="s" s="2">
         <v>77</v>
       </c>
@@ -6397,19 +6339,19 @@
         <v>77</v>
       </c>
       <c r="AB44" t="s" s="2">
-        <v>135</v>
+        <v>77</v>
       </c>
       <c r="AC44" t="s" s="2">
-        <v>189</v>
+        <v>77</v>
       </c>
       <c r="AD44" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AE44" t="s" s="2">
-        <v>136</v>
+        <v>77</v>
       </c>
       <c r="AF44" t="s" s="2">
-        <v>190</v>
+        <v>250</v>
       </c>
       <c r="AG44" t="s" s="2">
         <v>78</v>
@@ -6427,7 +6369,7 @@
         <v>77</v>
       </c>
       <c r="AL44" t="s" s="2">
-        <v>185</v>
+        <v>130</v>
       </c>
       <c r="AM44" t="s" s="2">
         <v>77</v>
@@ -6436,12 +6378,12 @@
         <v>77</v>
       </c>
     </row>
-    <row r="45" hidden="true">
+    <row r="45">
       <c r="A45" t="s" s="2">
-        <v>293</v>
+        <v>307</v>
       </c>
       <c r="B45" t="s" s="2">
-        <v>294</v>
+        <v>307</v>
       </c>
       <c r="C45" s="2"/>
       <c r="D45" t="s" s="2">
@@ -6452,32 +6394,28 @@
         <v>78</v>
       </c>
       <c r="G45" t="s" s="2">
-        <v>79</v>
+        <v>87</v>
       </c>
       <c r="H45" t="s" s="2">
-        <v>77</v>
+        <v>88</v>
       </c>
       <c r="I45" t="s" s="2">
         <v>77</v>
       </c>
       <c r="J45" t="s" s="2">
-        <v>88</v>
+        <v>77</v>
       </c>
       <c r="K45" t="s" s="2">
-        <v>192</v>
+        <v>181</v>
       </c>
       <c r="L45" t="s" s="2">
-        <v>295</v>
+        <v>308</v>
       </c>
       <c r="M45" t="s" s="2">
-        <v>194</v>
-      </c>
-      <c r="N45" t="s" s="2">
-        <v>195</v>
-      </c>
-      <c r="O45" t="s" s="2">
-        <v>196</v>
-      </c>
+        <v>309</v>
+      </c>
+      <c r="N45" s="2"/>
+      <c r="O45" s="2"/>
       <c r="P45" t="s" s="2">
         <v>77</v>
       </c>
@@ -6525,13 +6463,13 @@
         <v>77</v>
       </c>
       <c r="AF45" t="s" s="2">
-        <v>199</v>
+        <v>307</v>
       </c>
       <c r="AG45" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AH45" t="s" s="2">
-        <v>79</v>
+        <v>87</v>
       </c>
       <c r="AI45" t="s" s="2">
         <v>77</v>
@@ -6540,24 +6478,24 @@
         <v>99</v>
       </c>
       <c r="AK45" t="s" s="2">
-        <v>77</v>
+        <v>221</v>
       </c>
       <c r="AL45" t="s" s="2">
-        <v>200</v>
+        <v>166</v>
       </c>
       <c r="AM45" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AN45" t="s" s="2">
-        <v>201</v>
+        <v>310</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="s" s="2">
-        <v>296</v>
+        <v>311</v>
       </c>
       <c r="B46" t="s" s="2">
-        <v>297</v>
+        <v>311</v>
       </c>
       <c r="C46" s="2"/>
       <c r="D46" t="s" s="2">
@@ -6577,23 +6515,19 @@
         <v>77</v>
       </c>
       <c r="J46" t="s" s="2">
-        <v>88</v>
+        <v>77</v>
       </c>
       <c r="K46" t="s" s="2">
-        <v>181</v>
+        <v>312</v>
       </c>
       <c r="L46" t="s" s="2">
-        <v>298</v>
+        <v>313</v>
       </c>
       <c r="M46" t="s" s="2">
-        <v>204</v>
-      </c>
-      <c r="N46" t="s" s="2">
-        <v>205</v>
-      </c>
-      <c r="O46" t="s" s="2">
-        <v>206</v>
-      </c>
+        <v>314</v>
+      </c>
+      <c r="N46" s="2"/>
+      <c r="O46" s="2"/>
       <c r="P46" t="s" s="2">
         <v>77</v>
       </c>
@@ -6641,7 +6575,7 @@
         <v>77</v>
       </c>
       <c r="AF46" t="s" s="2">
-        <v>207</v>
+        <v>311</v>
       </c>
       <c r="AG46" t="s" s="2">
         <v>78</v>
@@ -6656,1374 +6590,20 @@
         <v>99</v>
       </c>
       <c r="AK46" t="s" s="2">
-        <v>77</v>
+        <v>221</v>
       </c>
       <c r="AL46" t="s" s="2">
-        <v>208</v>
+        <v>315</v>
       </c>
       <c r="AM46" t="s" s="2">
         <v>77</v>
       </c>
       <c r="AN46" t="s" s="2">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="47" hidden="true">
-      <c r="A47" t="s" s="2">
-        <v>299</v>
-      </c>
-      <c r="B47" t="s" s="2">
-        <v>259</v>
-      </c>
-      <c r="C47" s="2"/>
-      <c r="D47" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="E47" s="2"/>
-      <c r="F47" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="G47" t="s" s="2">
-        <v>87</v>
-      </c>
-      <c r="H47" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="I47" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="J47" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="K47" t="s" s="2">
-        <v>260</v>
-      </c>
-      <c r="L47" t="s" s="2">
-        <v>261</v>
-      </c>
-      <c r="M47" t="s" s="2">
-        <v>262</v>
-      </c>
-      <c r="N47" s="2"/>
-      <c r="O47" t="s" s="2">
-        <v>263</v>
-      </c>
-      <c r="P47" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="Q47" s="2"/>
-      <c r="R47" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="S47" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="T47" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="U47" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="V47" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="W47" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="X47" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="Y47" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="Z47" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AA47" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AB47" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AC47" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AD47" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AE47" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AF47" t="s" s="2">
-        <v>259</v>
-      </c>
-      <c r="AG47" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AH47" t="s" s="2">
-        <v>87</v>
-      </c>
-      <c r="AI47" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AJ47" t="s" s="2">
-        <v>99</v>
-      </c>
-      <c r="AK47" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AL47" t="s" s="2">
-        <v>264</v>
-      </c>
-      <c r="AM47" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AN47" t="s" s="2">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="s" s="2">
-        <v>300</v>
-      </c>
-      <c r="B48" t="s" s="2">
-        <v>265</v>
-      </c>
-      <c r="C48" s="2"/>
-      <c r="D48" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="E48" s="2"/>
-      <c r="F48" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="G48" t="s" s="2">
-        <v>87</v>
-      </c>
-      <c r="H48" t="s" s="2">
-        <v>88</v>
-      </c>
-      <c r="I48" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="J48" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="K48" t="s" s="2">
-        <v>234</v>
-      </c>
-      <c r="L48" t="s" s="2">
-        <v>301</v>
-      </c>
-      <c r="M48" t="s" s="2">
-        <v>267</v>
-      </c>
-      <c r="N48" s="2"/>
-      <c r="O48" s="2"/>
-      <c r="P48" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="Q48" s="2"/>
-      <c r="R48" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="S48" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="T48" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="U48" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="V48" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="W48" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="X48" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="Y48" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="Z48" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AA48" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AB48" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AC48" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AD48" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AE48" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AF48" t="s" s="2">
-        <v>265</v>
-      </c>
-      <c r="AG48" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AH48" t="s" s="2">
-        <v>87</v>
-      </c>
-      <c r="AI48" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AJ48" t="s" s="2">
-        <v>99</v>
-      </c>
-      <c r="AK48" t="s" s="2">
-        <v>268</v>
-      </c>
-      <c r="AL48" t="s" s="2">
-        <v>237</v>
-      </c>
-      <c r="AM48" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AN48" t="s" s="2">
-        <v>269</v>
-      </c>
-    </row>
-    <row r="49" hidden="true">
-      <c r="A49" t="s" s="2">
-        <v>302</v>
-      </c>
-      <c r="B49" t="s" s="2">
-        <v>303</v>
-      </c>
-      <c r="C49" s="2"/>
-      <c r="D49" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="E49" s="2"/>
-      <c r="F49" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="G49" t="s" s="2">
-        <v>87</v>
-      </c>
-      <c r="H49" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="I49" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="J49" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="K49" t="s" s="2">
-        <v>181</v>
-      </c>
-      <c r="L49" t="s" s="2">
-        <v>182</v>
-      </c>
-      <c r="M49" t="s" s="2">
-        <v>183</v>
-      </c>
-      <c r="N49" s="2"/>
-      <c r="O49" s="2"/>
-      <c r="P49" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="Q49" s="2"/>
-      <c r="R49" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="S49" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="T49" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="U49" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="V49" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="W49" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="X49" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="Y49" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="Z49" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AA49" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AB49" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AC49" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AD49" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AE49" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AF49" t="s" s="2">
-        <v>184</v>
-      </c>
-      <c r="AG49" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AH49" t="s" s="2">
-        <v>87</v>
-      </c>
-      <c r="AI49" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AJ49" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AK49" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AL49" t="s" s="2">
-        <v>185</v>
-      </c>
-      <c r="AM49" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AN49" t="s" s="2">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="50" hidden="true">
-      <c r="A50" t="s" s="2">
-        <v>304</v>
-      </c>
-      <c r="B50" t="s" s="2">
-        <v>305</v>
-      </c>
-      <c r="C50" s="2"/>
-      <c r="D50" t="s" s="2">
-        <v>155</v>
-      </c>
-      <c r="E50" s="2"/>
-      <c r="F50" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="G50" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="H50" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="I50" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="J50" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="K50" t="s" s="2">
-        <v>132</v>
-      </c>
-      <c r="L50" t="s" s="2">
-        <v>187</v>
-      </c>
-      <c r="M50" t="s" s="2">
-        <v>188</v>
-      </c>
-      <c r="N50" t="s" s="2">
-        <v>158</v>
-      </c>
-      <c r="O50" s="2"/>
-      <c r="P50" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="Q50" s="2"/>
-      <c r="R50" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="S50" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="T50" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="U50" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="V50" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="W50" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="X50" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="Y50" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="Z50" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AA50" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AB50" t="s" s="2">
-        <v>135</v>
-      </c>
-      <c r="AC50" t="s" s="2">
-        <v>189</v>
-      </c>
-      <c r="AD50" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AE50" t="s" s="2">
-        <v>136</v>
-      </c>
-      <c r="AF50" t="s" s="2">
-        <v>190</v>
-      </c>
-      <c r="AG50" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AH50" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AI50" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AJ50" t="s" s="2">
-        <v>138</v>
-      </c>
-      <c r="AK50" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AL50" t="s" s="2">
-        <v>185</v>
-      </c>
-      <c r="AM50" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AN50" t="s" s="2">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="s" s="2">
-        <v>306</v>
-      </c>
-      <c r="B51" t="s" s="2">
-        <v>307</v>
-      </c>
-      <c r="C51" s="2"/>
-      <c r="D51" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="E51" s="2"/>
-      <c r="F51" t="s" s="2">
-        <v>87</v>
-      </c>
-      <c r="G51" t="s" s="2">
-        <v>87</v>
-      </c>
-      <c r="H51" t="s" s="2">
-        <v>88</v>
-      </c>
-      <c r="I51" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="J51" t="s" s="2">
-        <v>88</v>
-      </c>
-      <c r="K51" t="s" s="2">
-        <v>308</v>
-      </c>
-      <c r="L51" t="s" s="2">
-        <v>309</v>
-      </c>
-      <c r="M51" t="s" s="2">
-        <v>310</v>
-      </c>
-      <c r="N51" s="2"/>
-      <c r="O51" s="2"/>
-      <c r="P51" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="Q51" s="2"/>
-      <c r="R51" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="S51" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="T51" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="U51" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="V51" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="W51" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="X51" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="Y51" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="Z51" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AA51" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AB51" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AC51" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AD51" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AE51" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AF51" t="s" s="2">
-        <v>311</v>
-      </c>
-      <c r="AG51" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AH51" t="s" s="2">
-        <v>87</v>
-      </c>
-      <c r="AI51" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AJ51" t="s" s="2">
-        <v>99</v>
-      </c>
-      <c r="AK51" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AL51" t="s" s="2">
-        <v>312</v>
-      </c>
-      <c r="AM51" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AN51" t="s" s="2">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="s" s="2">
-        <v>313</v>
-      </c>
-      <c r="B52" t="s" s="2">
-        <v>314</v>
-      </c>
-      <c r="C52" s="2"/>
-      <c r="D52" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="E52" s="2"/>
-      <c r="F52" t="s" s="2">
-        <v>87</v>
-      </c>
-      <c r="G52" t="s" s="2">
-        <v>87</v>
-      </c>
-      <c r="H52" t="s" s="2">
-        <v>88</v>
-      </c>
-      <c r="I52" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="J52" t="s" s="2">
-        <v>88</v>
-      </c>
-      <c r="K52" t="s" s="2">
-        <v>308</v>
-      </c>
-      <c r="L52" t="s" s="2">
-        <v>315</v>
-      </c>
-      <c r="M52" t="s" s="2">
         <v>316</v>
-      </c>
-      <c r="N52" s="2"/>
-      <c r="O52" s="2"/>
-      <c r="P52" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="Q52" s="2"/>
-      <c r="R52" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="S52" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="T52" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="U52" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="V52" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="W52" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="X52" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="Y52" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="Z52" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AA52" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AB52" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AC52" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AD52" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AE52" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AF52" t="s" s="2">
-        <v>317</v>
-      </c>
-      <c r="AG52" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AH52" t="s" s="2">
-        <v>87</v>
-      </c>
-      <c r="AI52" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AJ52" t="s" s="2">
-        <v>99</v>
-      </c>
-      <c r="AK52" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AL52" t="s" s="2">
-        <v>318</v>
-      </c>
-      <c r="AM52" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AN52" t="s" s="2">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="53" hidden="true">
-      <c r="A53" t="s" s="2">
-        <v>319</v>
-      </c>
-      <c r="B53" t="s" s="2">
-        <v>319</v>
-      </c>
-      <c r="C53" s="2"/>
-      <c r="D53" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="E53" s="2"/>
-      <c r="F53" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="G53" t="s" s="2">
-        <v>87</v>
-      </c>
-      <c r="H53" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="I53" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="J53" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="K53" t="s" s="2">
-        <v>239</v>
-      </c>
-      <c r="L53" t="s" s="2">
-        <v>320</v>
-      </c>
-      <c r="M53" t="s" s="2">
-        <v>321</v>
-      </c>
-      <c r="N53" s="2"/>
-      <c r="O53" s="2"/>
-      <c r="P53" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="Q53" s="2"/>
-      <c r="R53" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="S53" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="T53" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="U53" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="V53" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="W53" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="X53" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="Y53" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="Z53" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AA53" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AB53" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AC53" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AD53" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AE53" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AF53" t="s" s="2">
-        <v>319</v>
-      </c>
-      <c r="AG53" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AH53" t="s" s="2">
-        <v>87</v>
-      </c>
-      <c r="AI53" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AJ53" t="s" s="2">
-        <v>99</v>
-      </c>
-      <c r="AK53" t="s" s="2">
-        <v>221</v>
-      </c>
-      <c r="AL53" t="s" s="2">
-        <v>322</v>
-      </c>
-      <c r="AM53" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AN53" t="s" s="2">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="54" hidden="true">
-      <c r="A54" t="s" s="2">
-        <v>323</v>
-      </c>
-      <c r="B54" t="s" s="2">
-        <v>323</v>
-      </c>
-      <c r="C54" s="2"/>
-      <c r="D54" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="E54" s="2"/>
-      <c r="F54" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="G54" t="s" s="2">
-        <v>87</v>
-      </c>
-      <c r="H54" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="I54" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="J54" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="K54" t="s" s="2">
-        <v>181</v>
-      </c>
-      <c r="L54" t="s" s="2">
-        <v>182</v>
-      </c>
-      <c r="M54" t="s" s="2">
-        <v>183</v>
-      </c>
-      <c r="N54" s="2"/>
-      <c r="O54" s="2"/>
-      <c r="P54" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="Q54" s="2"/>
-      <c r="R54" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="S54" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="T54" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="U54" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="V54" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="W54" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="X54" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="Y54" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="Z54" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AA54" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AB54" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AC54" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AD54" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AE54" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AF54" t="s" s="2">
-        <v>184</v>
-      </c>
-      <c r="AG54" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AH54" t="s" s="2">
-        <v>87</v>
-      </c>
-      <c r="AI54" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AJ54" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AK54" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AL54" t="s" s="2">
-        <v>185</v>
-      </c>
-      <c r="AM54" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AN54" t="s" s="2">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="55" hidden="true">
-      <c r="A55" t="s" s="2">
-        <v>324</v>
-      </c>
-      <c r="B55" t="s" s="2">
-        <v>324</v>
-      </c>
-      <c r="C55" s="2"/>
-      <c r="D55" t="s" s="2">
-        <v>155</v>
-      </c>
-      <c r="E55" s="2"/>
-      <c r="F55" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="G55" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="H55" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="I55" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="J55" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="K55" t="s" s="2">
-        <v>132</v>
-      </c>
-      <c r="L55" t="s" s="2">
-        <v>187</v>
-      </c>
-      <c r="M55" t="s" s="2">
-        <v>188</v>
-      </c>
-      <c r="N55" t="s" s="2">
-        <v>158</v>
-      </c>
-      <c r="O55" s="2"/>
-      <c r="P55" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="Q55" s="2"/>
-      <c r="R55" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="S55" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="T55" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="U55" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="V55" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="W55" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="X55" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="Y55" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="Z55" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AA55" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AB55" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AC55" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AD55" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AE55" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AF55" t="s" s="2">
-        <v>190</v>
-      </c>
-      <c r="AG55" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AH55" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AI55" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AJ55" t="s" s="2">
-        <v>138</v>
-      </c>
-      <c r="AK55" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AL55" t="s" s="2">
-        <v>185</v>
-      </c>
-      <c r="AM55" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AN55" t="s" s="2">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="56" hidden="true">
-      <c r="A56" t="s" s="2">
-        <v>325</v>
-      </c>
-      <c r="B56" t="s" s="2">
-        <v>325</v>
-      </c>
-      <c r="C56" s="2"/>
-      <c r="D56" t="s" s="2">
-        <v>248</v>
-      </c>
-      <c r="E56" s="2"/>
-      <c r="F56" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="G56" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="H56" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="I56" t="s" s="2">
-        <v>88</v>
-      </c>
-      <c r="J56" t="s" s="2">
-        <v>88</v>
-      </c>
-      <c r="K56" t="s" s="2">
-        <v>132</v>
-      </c>
-      <c r="L56" t="s" s="2">
-        <v>249</v>
-      </c>
-      <c r="M56" t="s" s="2">
-        <v>250</v>
-      </c>
-      <c r="N56" t="s" s="2">
-        <v>158</v>
-      </c>
-      <c r="O56" t="s" s="2">
-        <v>159</v>
-      </c>
-      <c r="P56" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="Q56" s="2"/>
-      <c r="R56" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="S56" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="T56" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="U56" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="V56" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="W56" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="X56" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="Y56" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="Z56" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AA56" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AB56" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AC56" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AD56" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AE56" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AF56" t="s" s="2">
-        <v>251</v>
-      </c>
-      <c r="AG56" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AH56" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AI56" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AJ56" t="s" s="2">
-        <v>138</v>
-      </c>
-      <c r="AK56" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AL56" t="s" s="2">
-        <v>130</v>
-      </c>
-      <c r="AM56" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AN56" t="s" s="2">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="s" s="2">
-        <v>326</v>
-      </c>
-      <c r="B57" t="s" s="2">
-        <v>326</v>
-      </c>
-      <c r="C57" s="2"/>
-      <c r="D57" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="E57" s="2"/>
-      <c r="F57" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="G57" t="s" s="2">
-        <v>87</v>
-      </c>
-      <c r="H57" t="s" s="2">
-        <v>88</v>
-      </c>
-      <c r="I57" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="J57" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="K57" t="s" s="2">
-        <v>181</v>
-      </c>
-      <c r="L57" t="s" s="2">
-        <v>327</v>
-      </c>
-      <c r="M57" t="s" s="2">
-        <v>328</v>
-      </c>
-      <c r="N57" s="2"/>
-      <c r="O57" s="2"/>
-      <c r="P57" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="Q57" s="2"/>
-      <c r="R57" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="S57" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="T57" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="U57" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="V57" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="W57" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="X57" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="Y57" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="Z57" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AA57" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AB57" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AC57" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AD57" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AE57" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AF57" t="s" s="2">
-        <v>326</v>
-      </c>
-      <c r="AG57" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AH57" t="s" s="2">
-        <v>87</v>
-      </c>
-      <c r="AI57" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AJ57" t="s" s="2">
-        <v>99</v>
-      </c>
-      <c r="AK57" t="s" s="2">
-        <v>221</v>
-      </c>
-      <c r="AL57" t="s" s="2">
-        <v>166</v>
-      </c>
-      <c r="AM57" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AN57" t="s" s="2">
-        <v>329</v>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="s" s="2">
-        <v>330</v>
-      </c>
-      <c r="B58" t="s" s="2">
-        <v>330</v>
-      </c>
-      <c r="C58" s="2"/>
-      <c r="D58" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="E58" s="2"/>
-      <c r="F58" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="G58" t="s" s="2">
-        <v>87</v>
-      </c>
-      <c r="H58" t="s" s="2">
-        <v>88</v>
-      </c>
-      <c r="I58" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="J58" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="K58" t="s" s="2">
-        <v>331</v>
-      </c>
-      <c r="L58" t="s" s="2">
-        <v>332</v>
-      </c>
-      <c r="M58" t="s" s="2">
-        <v>333</v>
-      </c>
-      <c r="N58" s="2"/>
-      <c r="O58" s="2"/>
-      <c r="P58" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="Q58" s="2"/>
-      <c r="R58" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="S58" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="T58" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="U58" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="V58" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="W58" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="X58" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="Y58" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="Z58" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AA58" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AB58" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AC58" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AD58" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AE58" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AF58" t="s" s="2">
-        <v>330</v>
-      </c>
-      <c r="AG58" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AH58" t="s" s="2">
-        <v>87</v>
-      </c>
-      <c r="AI58" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AJ58" t="s" s="2">
-        <v>99</v>
-      </c>
-      <c r="AK58" t="s" s="2">
-        <v>221</v>
-      </c>
-      <c r="AL58" t="s" s="2">
-        <v>334</v>
-      </c>
-      <c r="AM58" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AN58" t="s" s="2">
-        <v>335</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AN58">
+  <autoFilter ref="A1:AN46">
     <filterColumn colId="7">
       <customFilters>
         <customFilter operator="notEqual" val=" "/>
@@ -8033,7 +6613,7 @@
       <filters blank="true"/>
     </filterColumn>
   </autoFilter>
-  <conditionalFormatting sqref="A2:AI57">
+  <conditionalFormatting sqref="A2:AI45">
     <cfRule type="expression" dxfId="0" priority="1">
       <formula>$G2&lt;&gt;"Y"</formula>
     </cfRule>

</xml_diff>